<commit_message>
chore(dev): run the frontend on 3001 so it pairs with the backend on 8001
The backend moved to 8001; leaving Next on 3000 meant every local session
started with a port clash against whatever else was already bound there.
The Class 10 queue sheet carries the status the overnight runner wrote back.

Co-Authored-By: Claude Opus 5 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/backend/queue/class10_cbse_queue.xlsx
+++ b/backend/queue/class10_cbse_queue.xlsx
@@ -1,13 +1,13 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="queue" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="queue" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'queue'!$A$1:$S$1</definedName>
@@ -600,14 +600,33 @@
       </c>
       <c r="K2" t="inlineStr">
         <is>
-          <t>pending</t>
-        </is>
+          <t>done</t>
+        </is>
+      </c>
+      <c r="L2" t="n">
+        <v>333</v>
+      </c>
+      <c r="M2" t="n">
+        <v>12</v>
+      </c>
+      <c r="N2" t="n">
+        <v>29282</v>
+      </c>
+      <c r="O2" t="n">
+        <v>16</v>
+      </c>
+      <c r="P2" t="n">
+        <v>690.5</v>
       </c>
       <c r="Q2" t="n">
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="R2" t="inlineStr"/>
-      <c r="S2" t="inlineStr"/>
+      <c r="S2" t="inlineStr">
+        <is>
+          <t>2026-09-19T01:55:10</t>
+        </is>
+      </c>
     </row>
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
@@ -654,19 +673,33 @@
       </c>
       <c r="K3" s="2" t="inlineStr">
         <is>
-          <t>pending</t>
-        </is>
-      </c>
-      <c r="L3" s="2" t="n"/>
-      <c r="M3" s="2" t="n"/>
-      <c r="N3" s="2" t="n"/>
-      <c r="O3" s="2" t="n"/>
-      <c r="P3" s="2" t="n"/>
+          <t>done</t>
+        </is>
+      </c>
+      <c r="L3" s="2" t="n">
+        <v>234</v>
+      </c>
+      <c r="M3" s="2" t="n">
+        <v>6</v>
+      </c>
+      <c r="N3" s="2" t="n">
+        <v>13172</v>
+      </c>
+      <c r="O3" s="2" t="n">
+        <v>6</v>
+      </c>
+      <c r="P3" s="2" t="n">
+        <v>157.1</v>
+      </c>
       <c r="Q3" s="2" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="R3" s="2" t="inlineStr"/>
-      <c r="S3" s="2" t="inlineStr"/>
+      <c r="S3" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-18T18:42:42</t>
+        </is>
+      </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -713,14 +746,32 @@
       </c>
       <c r="K4" t="inlineStr">
         <is>
-          <t>pending</t>
-        </is>
+          <t>done</t>
+        </is>
+      </c>
+      <c r="L4" t="n">
+        <v>213</v>
+      </c>
+      <c r="M4" t="n">
+        <v>11</v>
+      </c>
+      <c r="N4" t="n">
+        <v>25449</v>
+      </c>
+      <c r="O4" t="n">
+        <v>16</v>
+      </c>
+      <c r="P4" t="n">
+        <v>2769.9</v>
       </c>
       <c r="Q4" t="n">
-        <v>0</v>
-      </c>
-      <c r="R4" t="inlineStr"/>
-      <c r="S4" t="inlineStr"/>
+        <v>1</v>
+      </c>
+      <c r="S4" t="inlineStr">
+        <is>
+          <t>2026-09-17T23:34:08</t>
+        </is>
+      </c>
     </row>
     <row r="5">
       <c r="A5" s="2" t="inlineStr">
@@ -767,19 +818,33 @@
       </c>
       <c r="K5" s="2" t="inlineStr">
         <is>
-          <t>pending</t>
-        </is>
-      </c>
-      <c r="L5" s="2" t="n"/>
-      <c r="M5" s="2" t="n"/>
-      <c r="N5" s="2" t="n"/>
-      <c r="O5" s="2" t="n"/>
-      <c r="P5" s="2" t="n"/>
+          <t>done</t>
+        </is>
+      </c>
+      <c r="L5" s="2" t="n">
+        <v>235</v>
+      </c>
+      <c r="M5" s="2" t="n">
+        <v>12</v>
+      </c>
+      <c r="N5" s="2" t="n">
+        <v>26806</v>
+      </c>
+      <c r="O5" s="2" t="n">
+        <v>20</v>
+      </c>
+      <c r="P5" s="2" t="n">
+        <v>706.5</v>
+      </c>
       <c r="Q5" s="2" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="R5" s="2" t="inlineStr"/>
-      <c r="S5" s="2" t="inlineStr"/>
+      <c r="S5" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-18T18:55:06</t>
+        </is>
+      </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
@@ -826,14 +891,32 @@
       </c>
       <c r="K6" t="inlineStr">
         <is>
-          <t>pending</t>
-        </is>
+          <t>done</t>
+        </is>
+      </c>
+      <c r="L6" t="n">
+        <v>237</v>
+      </c>
+      <c r="M6" t="n">
+        <v>16</v>
+      </c>
+      <c r="N6" t="n">
+        <v>38654</v>
+      </c>
+      <c r="O6" t="n">
+        <v>20</v>
+      </c>
+      <c r="P6" t="n">
+        <v>209.7</v>
       </c>
       <c r="Q6" t="n">
-        <v>0</v>
-      </c>
-      <c r="R6" t="inlineStr"/>
-      <c r="S6" t="inlineStr"/>
+        <v>2</v>
+      </c>
+      <c r="S6" t="inlineStr">
+        <is>
+          <t>2026-09-18T18:58:36</t>
+        </is>
+      </c>
     </row>
     <row r="7">
       <c r="A7" s="2" t="inlineStr">
@@ -880,19 +963,33 @@
       </c>
       <c r="K7" s="2" t="inlineStr">
         <is>
-          <t>pending</t>
-        </is>
-      </c>
-      <c r="L7" s="2" t="n"/>
-      <c r="M7" s="2" t="n"/>
-      <c r="N7" s="2" t="n"/>
-      <c r="O7" s="2" t="n"/>
-      <c r="P7" s="2" t="n"/>
+          <t>done</t>
+        </is>
+      </c>
+      <c r="L7" s="2" t="n">
+        <v>238</v>
+      </c>
+      <c r="M7" s="2" t="n">
+        <v>13</v>
+      </c>
+      <c r="N7" s="2" t="n">
+        <v>26650</v>
+      </c>
+      <c r="O7" s="2" t="n">
+        <v>12</v>
+      </c>
+      <c r="P7" s="2" t="n">
+        <v>528.5</v>
+      </c>
       <c r="Q7" s="2" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="R7" s="2" t="inlineStr"/>
-      <c r="S7" s="2" t="inlineStr"/>
+      <c r="S7" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-18T19:07:25</t>
+        </is>
+      </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
@@ -939,14 +1036,32 @@
       </c>
       <c r="K8" t="inlineStr">
         <is>
-          <t>pending</t>
-        </is>
+          <t>done</t>
+        </is>
+      </c>
+      <c r="L8" t="n">
+        <v>239</v>
+      </c>
+      <c r="M8" t="n">
+        <v>13</v>
+      </c>
+      <c r="N8" t="n">
+        <v>28477</v>
+      </c>
+      <c r="O8" t="n">
+        <v>17</v>
+      </c>
+      <c r="P8" t="n">
+        <v>774.3</v>
       </c>
       <c r="Q8" t="n">
-        <v>0</v>
-      </c>
-      <c r="R8" t="inlineStr"/>
-      <c r="S8" t="inlineStr"/>
+        <v>2</v>
+      </c>
+      <c r="S8" t="inlineStr">
+        <is>
+          <t>2026-09-18T19:20:21</t>
+        </is>
+      </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
@@ -993,14 +1108,32 @@
       </c>
       <c r="K9" t="inlineStr">
         <is>
-          <t>pending</t>
-        </is>
+          <t>done</t>
+        </is>
+      </c>
+      <c r="L9" t="n">
+        <v>241</v>
+      </c>
+      <c r="M9" t="n">
+        <v>16</v>
+      </c>
+      <c r="N9" t="n">
+        <v>37341</v>
+      </c>
+      <c r="O9" t="n">
+        <v>25</v>
+      </c>
+      <c r="P9" t="n">
+        <v>1520.9</v>
       </c>
       <c r="Q9" t="n">
-        <v>0</v>
-      </c>
-      <c r="R9" t="inlineStr"/>
-      <c r="S9" t="inlineStr"/>
+        <v>2</v>
+      </c>
+      <c r="S9" t="inlineStr">
+        <is>
+          <t>2026-09-18T19:45:43</t>
+        </is>
+      </c>
     </row>
     <row r="10">
       <c r="A10" s="2" t="inlineStr">
@@ -1047,19 +1180,33 @@
       </c>
       <c r="K10" s="2" t="inlineStr">
         <is>
-          <t>pending</t>
-        </is>
-      </c>
-      <c r="L10" s="2" t="n"/>
-      <c r="M10" s="2" t="n"/>
-      <c r="N10" s="2" t="n"/>
-      <c r="O10" s="2" t="n"/>
-      <c r="P10" s="2" t="n"/>
+          <t>done</t>
+        </is>
+      </c>
+      <c r="L10" s="2" t="n">
+        <v>242</v>
+      </c>
+      <c r="M10" s="2" t="n">
+        <v>20</v>
+      </c>
+      <c r="N10" s="2" t="n">
+        <v>49017</v>
+      </c>
+      <c r="O10" s="2" t="n">
+        <v>24</v>
+      </c>
+      <c r="P10" s="2" t="n">
+        <v>1181.8</v>
+      </c>
       <c r="Q10" s="2" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="R10" s="2" t="inlineStr"/>
-      <c r="S10" s="2" t="inlineStr"/>
+      <c r="S10" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-18T19:40:04</t>
+        </is>
+      </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
@@ -1106,14 +1253,32 @@
       </c>
       <c r="K11" t="inlineStr">
         <is>
-          <t>pending</t>
-        </is>
+          <t>done</t>
+        </is>
+      </c>
+      <c r="L11" t="n">
+        <v>243</v>
+      </c>
+      <c r="M11" t="n">
+        <v>16</v>
+      </c>
+      <c r="N11" t="n">
+        <v>36518</v>
+      </c>
+      <c r="O11" t="n">
+        <v>29</v>
+      </c>
+      <c r="P11" t="n">
+        <v>416.5</v>
       </c>
       <c r="Q11" t="n">
-        <v>0</v>
-      </c>
-      <c r="R11" t="inlineStr"/>
-      <c r="S11" t="inlineStr"/>
+        <v>1</v>
+      </c>
+      <c r="S11" t="inlineStr">
+        <is>
+          <t>2026-09-18T19:52:41</t>
+        </is>
+      </c>
     </row>
     <row r="12">
       <c r="A12" s="2" t="inlineStr">
@@ -1160,19 +1325,33 @@
       </c>
       <c r="K12" s="2" t="inlineStr">
         <is>
-          <t>pending</t>
-        </is>
-      </c>
-      <c r="L12" s="2" t="n"/>
-      <c r="M12" s="2" t="n"/>
-      <c r="N12" s="2" t="n"/>
-      <c r="O12" s="2" t="n"/>
-      <c r="P12" s="2" t="n"/>
+          <t>done</t>
+        </is>
+      </c>
+      <c r="L12" s="2" t="n">
+        <v>250</v>
+      </c>
+      <c r="M12" s="2" t="n">
+        <v>20</v>
+      </c>
+      <c r="N12" s="2" t="n">
+        <v>43572</v>
+      </c>
+      <c r="O12" s="2" t="n">
+        <v>21</v>
+      </c>
+      <c r="P12" s="2" t="n">
+        <v>381.3</v>
+      </c>
       <c r="Q12" s="2" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="R12" s="2" t="inlineStr"/>
-      <c r="S12" s="2" t="inlineStr"/>
+      <c r="S12" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-18T19:59:04</t>
+        </is>
+      </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
@@ -1219,14 +1398,32 @@
       </c>
       <c r="K13" t="inlineStr">
         <is>
-          <t>pending</t>
-        </is>
+          <t>done</t>
+        </is>
+      </c>
+      <c r="L13" t="n">
+        <v>251</v>
+      </c>
+      <c r="M13" t="n">
+        <v>19</v>
+      </c>
+      <c r="N13" t="n">
+        <v>52212</v>
+      </c>
+      <c r="O13" t="n">
+        <v>28</v>
+      </c>
+      <c r="P13" t="n">
+        <v>2371.1</v>
       </c>
       <c r="Q13" t="n">
-        <v>0</v>
-      </c>
-      <c r="R13" t="inlineStr"/>
-      <c r="S13" t="inlineStr"/>
+        <v>1</v>
+      </c>
+      <c r="S13" t="inlineStr">
+        <is>
+          <t>2026-09-18T20:38:36</t>
+        </is>
+      </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
@@ -1273,14 +1470,32 @@
       </c>
       <c r="K14" t="inlineStr">
         <is>
-          <t>pending</t>
-        </is>
+          <t>done</t>
+        </is>
+      </c>
+      <c r="L14" t="n">
+        <v>262</v>
+      </c>
+      <c r="M14" t="n">
+        <v>27</v>
+      </c>
+      <c r="N14" t="n">
+        <v>55322</v>
+      </c>
+      <c r="O14" t="n">
+        <v>25</v>
+      </c>
+      <c r="P14" t="n">
+        <v>298.8</v>
       </c>
       <c r="Q14" t="n">
-        <v>0</v>
-      </c>
-      <c r="R14" t="inlineStr"/>
-      <c r="S14" t="inlineStr"/>
+        <v>1</v>
+      </c>
+      <c r="S14" t="inlineStr">
+        <is>
+          <t>2026-09-18T20:43:36</t>
+        </is>
+      </c>
     </row>
     <row r="15">
       <c r="A15" s="2" t="inlineStr">
@@ -1327,19 +1542,33 @@
       </c>
       <c r="K15" s="2" t="inlineStr">
         <is>
-          <t>pending</t>
-        </is>
-      </c>
-      <c r="L15" s="2" t="n"/>
-      <c r="M15" s="2" t="n"/>
-      <c r="N15" s="2" t="n"/>
-      <c r="O15" s="2" t="n"/>
-      <c r="P15" s="2" t="n"/>
+          <t>done</t>
+        </is>
+      </c>
+      <c r="L15" s="2" t="n">
+        <v>263</v>
+      </c>
+      <c r="M15" s="2" t="n">
+        <v>22</v>
+      </c>
+      <c r="N15" s="2" t="n">
+        <v>51902</v>
+      </c>
+      <c r="O15" s="2" t="n">
+        <v>16</v>
+      </c>
+      <c r="P15" s="2" t="n">
+        <v>321.5</v>
+      </c>
       <c r="Q15" s="2" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="R15" s="2" t="inlineStr"/>
-      <c r="S15" s="2" t="inlineStr"/>
+      <c r="S15" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-18T20:48:59</t>
+        </is>
+      </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
@@ -1386,14 +1615,32 @@
       </c>
       <c r="K16" t="inlineStr">
         <is>
-          <t>pending</t>
-        </is>
+          <t>done</t>
+        </is>
+      </c>
+      <c r="L16" t="n">
+        <v>264</v>
+      </c>
+      <c r="M16" t="n">
+        <v>27</v>
+      </c>
+      <c r="N16" t="n">
+        <v>57027</v>
+      </c>
+      <c r="O16" t="n">
+        <v>27</v>
+      </c>
+      <c r="P16" t="n">
+        <v>231.3</v>
       </c>
       <c r="Q16" t="n">
-        <v>0</v>
-      </c>
-      <c r="R16" t="inlineStr"/>
-      <c r="S16" t="inlineStr"/>
+        <v>1</v>
+      </c>
+      <c r="S16" t="inlineStr">
+        <is>
+          <t>2026-09-18T20:52:52</t>
+        </is>
+      </c>
     </row>
     <row r="17">
       <c r="A17" s="2" t="inlineStr">
@@ -1440,19 +1687,33 @@
       </c>
       <c r="K17" s="2" t="inlineStr">
         <is>
-          <t>pending</t>
-        </is>
-      </c>
-      <c r="L17" s="2" t="n"/>
-      <c r="M17" s="2" t="n"/>
-      <c r="N17" s="2" t="n"/>
-      <c r="O17" s="2" t="n"/>
-      <c r="P17" s="2" t="n"/>
+          <t>done</t>
+        </is>
+      </c>
+      <c r="L17" s="2" t="n">
+        <v>265</v>
+      </c>
+      <c r="M17" s="2" t="n">
+        <v>24</v>
+      </c>
+      <c r="N17" s="2" t="n">
+        <v>50541</v>
+      </c>
+      <c r="O17" s="2" t="n">
+        <v>29</v>
+      </c>
+      <c r="P17" s="2" t="n">
+        <v>200.1</v>
+      </c>
       <c r="Q17" s="2" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="R17" s="2" t="inlineStr"/>
-      <c r="S17" s="2" t="inlineStr"/>
+      <c r="S17" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-18T20:56:13</t>
+        </is>
+      </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
@@ -1499,14 +1760,32 @@
       </c>
       <c r="K18" t="inlineStr">
         <is>
-          <t>pending</t>
-        </is>
+          <t>done</t>
+        </is>
+      </c>
+      <c r="L18" t="n">
+        <v>266</v>
+      </c>
+      <c r="M18" t="n">
+        <v>25</v>
+      </c>
+      <c r="N18" t="n">
+        <v>55919</v>
+      </c>
+      <c r="O18" t="n">
+        <v>26</v>
+      </c>
+      <c r="P18" t="n">
+        <v>226.5</v>
       </c>
       <c r="Q18" t="n">
-        <v>0</v>
-      </c>
-      <c r="R18" t="inlineStr"/>
-      <c r="S18" t="inlineStr"/>
+        <v>1</v>
+      </c>
+      <c r="S18" t="inlineStr">
+        <is>
+          <t>2026-09-18T21:00:00</t>
+        </is>
+      </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
@@ -1553,14 +1832,32 @@
       </c>
       <c r="K19" t="inlineStr">
         <is>
-          <t>pending</t>
-        </is>
+          <t>done</t>
+        </is>
+      </c>
+      <c r="L19" t="n">
+        <v>267</v>
+      </c>
+      <c r="M19" t="n">
+        <v>12</v>
+      </c>
+      <c r="N19" t="n">
+        <v>27740</v>
+      </c>
+      <c r="O19" t="n">
+        <v>17</v>
+      </c>
+      <c r="P19" t="n">
+        <v>338.2</v>
       </c>
       <c r="Q19" t="n">
-        <v>0</v>
-      </c>
-      <c r="R19" t="inlineStr"/>
-      <c r="S19" t="inlineStr"/>
+        <v>1</v>
+      </c>
+      <c r="S19" t="inlineStr">
+        <is>
+          <t>2026-09-18T21:05:39</t>
+        </is>
+      </c>
     </row>
     <row r="20">
       <c r="A20" s="2" t="inlineStr">
@@ -1607,19 +1904,33 @@
       </c>
       <c r="K20" s="2" t="inlineStr">
         <is>
-          <t>pending</t>
-        </is>
-      </c>
-      <c r="L20" s="2" t="n"/>
-      <c r="M20" s="2" t="n"/>
-      <c r="N20" s="2" t="n"/>
-      <c r="O20" s="2" t="n"/>
-      <c r="P20" s="2" t="n"/>
+          <t>done</t>
+        </is>
+      </c>
+      <c r="L20" s="2" t="n">
+        <v>268</v>
+      </c>
+      <c r="M20" s="2" t="n">
+        <v>16</v>
+      </c>
+      <c r="N20" s="2" t="n">
+        <v>36058</v>
+      </c>
+      <c r="O20" s="2" t="n">
+        <v>20</v>
+      </c>
+      <c r="P20" s="2" t="n">
+        <v>485.1</v>
+      </c>
       <c r="Q20" s="2" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="R20" s="2" t="inlineStr"/>
-      <c r="S20" s="2" t="inlineStr"/>
+      <c r="S20" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-18T21:13:45</t>
+        </is>
+      </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
@@ -1666,14 +1977,32 @@
       </c>
       <c r="K21" t="inlineStr">
         <is>
-          <t>pending</t>
-        </is>
+          <t>done</t>
+        </is>
+      </c>
+      <c r="L21" t="n">
+        <v>269</v>
+      </c>
+      <c r="M21" t="n">
+        <v>17</v>
+      </c>
+      <c r="N21" t="n">
+        <v>34919</v>
+      </c>
+      <c r="O21" t="n">
+        <v>18</v>
+      </c>
+      <c r="P21" t="n">
+        <v>509.3</v>
       </c>
       <c r="Q21" t="n">
-        <v>0</v>
-      </c>
-      <c r="R21" t="inlineStr"/>
-      <c r="S21" t="inlineStr"/>
+        <v>1</v>
+      </c>
+      <c r="S21" t="inlineStr">
+        <is>
+          <t>2026-09-18T21:22:15</t>
+        </is>
+      </c>
     </row>
     <row r="22">
       <c r="A22" s="2" t="inlineStr">
@@ -1720,19 +2049,33 @@
       </c>
       <c r="K22" s="2" t="inlineStr">
         <is>
-          <t>pending</t>
-        </is>
-      </c>
-      <c r="L22" s="2" t="n"/>
-      <c r="M22" s="2" t="n"/>
-      <c r="N22" s="2" t="n"/>
-      <c r="O22" s="2" t="n"/>
-      <c r="P22" s="2" t="n"/>
+          <t>done</t>
+        </is>
+      </c>
+      <c r="L22" s="2" t="n">
+        <v>270</v>
+      </c>
+      <c r="M22" s="2" t="n">
+        <v>17</v>
+      </c>
+      <c r="N22" s="2" t="n">
+        <v>37011</v>
+      </c>
+      <c r="O22" s="2" t="n">
+        <v>23</v>
+      </c>
+      <c r="P22" s="2" t="n">
+        <v>333.4</v>
+      </c>
       <c r="Q22" s="2" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="R22" s="2" t="inlineStr"/>
-      <c r="S22" s="2" t="inlineStr"/>
+      <c r="S22" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-18T21:27:49</t>
+        </is>
+      </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
@@ -1779,14 +2122,32 @@
       </c>
       <c r="K23" t="inlineStr">
         <is>
-          <t>pending</t>
-        </is>
+          <t>done</t>
+        </is>
+      </c>
+      <c r="L23" t="n">
+        <v>271</v>
+      </c>
+      <c r="M23" t="n">
+        <v>12</v>
+      </c>
+      <c r="N23" t="n">
+        <v>24135</v>
+      </c>
+      <c r="O23" t="n">
+        <v>18</v>
+      </c>
+      <c r="P23" t="n">
+        <v>345</v>
       </c>
       <c r="Q23" t="n">
-        <v>0</v>
-      </c>
-      <c r="R23" t="inlineStr"/>
-      <c r="S23" t="inlineStr"/>
+        <v>1</v>
+      </c>
+      <c r="S23" t="inlineStr">
+        <is>
+          <t>2026-09-18T21:33:35</t>
+        </is>
+      </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
@@ -1833,14 +2194,32 @@
       </c>
       <c r="K24" t="inlineStr">
         <is>
-          <t>pending</t>
-        </is>
+          <t>done</t>
+        </is>
+      </c>
+      <c r="L24" t="n">
+        <v>272</v>
+      </c>
+      <c r="M24" t="n">
+        <v>15</v>
+      </c>
+      <c r="N24" t="n">
+        <v>22015</v>
+      </c>
+      <c r="O24" t="n">
+        <v>6</v>
+      </c>
+      <c r="P24" t="n">
+        <v>269.7</v>
       </c>
       <c r="Q24" t="n">
-        <v>0</v>
-      </c>
-      <c r="R24" t="inlineStr"/>
-      <c r="S24" t="inlineStr"/>
+        <v>1</v>
+      </c>
+      <c r="S24" t="inlineStr">
+        <is>
+          <t>2026-09-18T21:38:06</t>
+        </is>
+      </c>
     </row>
     <row r="25">
       <c r="A25" s="2" t="inlineStr">
@@ -1887,19 +2266,33 @@
       </c>
       <c r="K25" s="2" t="inlineStr">
         <is>
-          <t>pending</t>
-        </is>
-      </c>
-      <c r="L25" s="2" t="n"/>
-      <c r="M25" s="2" t="n"/>
-      <c r="N25" s="2" t="n"/>
-      <c r="O25" s="2" t="n"/>
-      <c r="P25" s="2" t="n"/>
+          <t>done</t>
+        </is>
+      </c>
+      <c r="L25" s="2" t="n">
+        <v>273</v>
+      </c>
+      <c r="M25" s="2" t="n">
+        <v>16</v>
+      </c>
+      <c r="N25" s="2" t="n">
+        <v>26475</v>
+      </c>
+      <c r="O25" s="2" t="n">
+        <v>11</v>
+      </c>
+      <c r="P25" s="2" t="n">
+        <v>327.7</v>
+      </c>
       <c r="Q25" s="2" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="R25" s="2" t="inlineStr"/>
-      <c r="S25" s="2" t="inlineStr"/>
+      <c r="S25" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-18T21:43:34</t>
+        </is>
+      </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
@@ -1946,14 +2339,32 @@
       </c>
       <c r="K26" t="inlineStr">
         <is>
-          <t>pending</t>
-        </is>
+          <t>done</t>
+        </is>
+      </c>
+      <c r="L26" t="n">
+        <v>274</v>
+      </c>
+      <c r="M26" t="n">
+        <v>16</v>
+      </c>
+      <c r="N26" t="n">
+        <v>22844</v>
+      </c>
+      <c r="O26" t="n">
+        <v>16</v>
+      </c>
+      <c r="P26" t="n">
+        <v>213.1</v>
       </c>
       <c r="Q26" t="n">
-        <v>0</v>
-      </c>
-      <c r="R26" t="inlineStr"/>
-      <c r="S26" t="inlineStr"/>
+        <v>1</v>
+      </c>
+      <c r="S26" t="inlineStr">
+        <is>
+          <t>2026-09-18T21:47:08</t>
+        </is>
+      </c>
     </row>
     <row r="27">
       <c r="A27" s="2" t="inlineStr">
@@ -2000,19 +2411,33 @@
       </c>
       <c r="K27" s="2" t="inlineStr">
         <is>
-          <t>pending</t>
-        </is>
-      </c>
-      <c r="L27" s="2" t="n"/>
-      <c r="M27" s="2" t="n"/>
-      <c r="N27" s="2" t="n"/>
-      <c r="O27" s="2" t="n"/>
-      <c r="P27" s="2" t="n"/>
+          <t>done</t>
+        </is>
+      </c>
+      <c r="L27" s="2" t="n">
+        <v>275</v>
+      </c>
+      <c r="M27" s="2" t="n">
+        <v>15</v>
+      </c>
+      <c r="N27" s="2" t="n">
+        <v>26632</v>
+      </c>
+      <c r="O27" s="2" t="n">
+        <v>3</v>
+      </c>
+      <c r="P27" s="2" t="n">
+        <v>291.6</v>
+      </c>
       <c r="Q27" s="2" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="R27" s="2" t="inlineStr"/>
-      <c r="S27" s="2" t="inlineStr"/>
+      <c r="S27" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-18T21:52:00</t>
+        </is>
+      </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
@@ -2059,14 +2484,32 @@
       </c>
       <c r="K28" t="inlineStr">
         <is>
-          <t>pending</t>
-        </is>
+          <t>done</t>
+        </is>
+      </c>
+      <c r="L28" t="n">
+        <v>276</v>
+      </c>
+      <c r="M28" t="n">
+        <v>17</v>
+      </c>
+      <c r="N28" t="n">
+        <v>28410</v>
+      </c>
+      <c r="O28" t="n">
+        <v>7</v>
+      </c>
+      <c r="P28" t="n">
+        <v>200.9</v>
       </c>
       <c r="Q28" t="n">
-        <v>0</v>
-      </c>
-      <c r="R28" t="inlineStr"/>
-      <c r="S28" t="inlineStr"/>
+        <v>1</v>
+      </c>
+      <c r="S28" t="inlineStr">
+        <is>
+          <t>2026-09-18T21:55:22</t>
+        </is>
+      </c>
     </row>
     <row r="29">
       <c r="A29" s="2" t="inlineStr">
@@ -2113,19 +2556,33 @@
       </c>
       <c r="K29" s="2" t="inlineStr">
         <is>
-          <t>pending</t>
-        </is>
-      </c>
-      <c r="L29" s="2" t="n"/>
-      <c r="M29" s="2" t="n"/>
-      <c r="N29" s="2" t="n"/>
-      <c r="O29" s="2" t="n"/>
-      <c r="P29" s="2" t="n"/>
+          <t>done</t>
+        </is>
+      </c>
+      <c r="L29" s="2" t="n">
+        <v>277</v>
+      </c>
+      <c r="M29" s="2" t="n">
+        <v>14</v>
+      </c>
+      <c r="N29" s="2" t="n">
+        <v>24722</v>
+      </c>
+      <c r="O29" s="2" t="n">
+        <v>5</v>
+      </c>
+      <c r="P29" s="2" t="n">
+        <v>265.8</v>
+      </c>
       <c r="Q29" s="2" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="R29" s="2" t="inlineStr"/>
-      <c r="S29" s="2" t="inlineStr"/>
+      <c r="S29" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-18T21:59:49</t>
+        </is>
+      </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
@@ -2172,14 +2629,32 @@
       </c>
       <c r="K30" t="inlineStr">
         <is>
-          <t>pending</t>
-        </is>
+          <t>done</t>
+        </is>
+      </c>
+      <c r="L30" t="n">
+        <v>278</v>
+      </c>
+      <c r="M30" t="n">
+        <v>17</v>
+      </c>
+      <c r="N30" t="n">
+        <v>25613</v>
+      </c>
+      <c r="O30" t="n">
+        <v>5</v>
+      </c>
+      <c r="P30" t="n">
+        <v>367.7</v>
       </c>
       <c r="Q30" t="n">
-        <v>0</v>
-      </c>
-      <c r="R30" t="inlineStr"/>
-      <c r="S30" t="inlineStr"/>
+        <v>1</v>
+      </c>
+      <c r="S30" t="inlineStr">
+        <is>
+          <t>2026-09-18T22:05:58</t>
+        </is>
+      </c>
     </row>
     <row r="31">
       <c r="A31" s="2" t="inlineStr">
@@ -2226,19 +2701,33 @@
       </c>
       <c r="K31" s="2" t="inlineStr">
         <is>
-          <t>pending</t>
-        </is>
-      </c>
-      <c r="L31" s="2" t="n"/>
-      <c r="M31" s="2" t="n"/>
-      <c r="N31" s="2" t="n"/>
-      <c r="O31" s="2" t="n"/>
-      <c r="P31" s="2" t="n"/>
+          <t>done</t>
+        </is>
+      </c>
+      <c r="L31" s="2" t="n">
+        <v>279</v>
+      </c>
+      <c r="M31" s="2" t="n">
+        <v>9</v>
+      </c>
+      <c r="N31" s="2" t="n">
+        <v>15752</v>
+      </c>
+      <c r="O31" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="P31" s="2" t="n">
+        <v>230.2</v>
+      </c>
       <c r="Q31" s="2" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="R31" s="2" t="inlineStr"/>
-      <c r="S31" s="2" t="inlineStr"/>
+      <c r="S31" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-18T22:09:49</t>
+        </is>
+      </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
@@ -2285,14 +2774,32 @@
       </c>
       <c r="K32" t="inlineStr">
         <is>
-          <t>pending</t>
-        </is>
+          <t>done</t>
+        </is>
+      </c>
+      <c r="L32" t="n">
+        <v>280</v>
+      </c>
+      <c r="M32" t="n">
+        <v>21</v>
+      </c>
+      <c r="N32" t="n">
+        <v>39465</v>
+      </c>
+      <c r="O32" t="n">
+        <v>6</v>
+      </c>
+      <c r="P32" t="n">
+        <v>471.1</v>
       </c>
       <c r="Q32" t="n">
-        <v>0</v>
-      </c>
-      <c r="R32" t="inlineStr"/>
-      <c r="S32" t="inlineStr"/>
+        <v>1</v>
+      </c>
+      <c r="S32" t="inlineStr">
+        <is>
+          <t>2026-09-18T22:17:41</t>
+        </is>
+      </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
@@ -2339,14 +2846,32 @@
       </c>
       <c r="K33" t="inlineStr">
         <is>
-          <t>pending</t>
-        </is>
+          <t>done</t>
+        </is>
+      </c>
+      <c r="L33" t="n">
+        <v>281</v>
+      </c>
+      <c r="M33" t="n">
+        <v>7</v>
+      </c>
+      <c r="N33" t="n">
+        <v>11586</v>
+      </c>
+      <c r="O33" t="n">
+        <v>6</v>
+      </c>
+      <c r="P33" t="n">
+        <v>119.1</v>
       </c>
       <c r="Q33" t="n">
-        <v>0</v>
-      </c>
-      <c r="R33" t="inlineStr"/>
-      <c r="S33" t="inlineStr"/>
+        <v>1</v>
+      </c>
+      <c r="S33" t="inlineStr">
+        <is>
+          <t>2026-09-18T22:19:41</t>
+        </is>
+      </c>
     </row>
     <row r="34">
       <c r="A34" s="2" t="inlineStr">
@@ -2393,19 +2918,33 @@
       </c>
       <c r="K34" s="2" t="inlineStr">
         <is>
-          <t>pending</t>
-        </is>
-      </c>
-      <c r="L34" s="2" t="n"/>
-      <c r="M34" s="2" t="n"/>
-      <c r="N34" s="2" t="n"/>
-      <c r="O34" s="2" t="n"/>
-      <c r="P34" s="2" t="n"/>
+          <t>done</t>
+        </is>
+      </c>
+      <c r="L34" s="2" t="n">
+        <v>282</v>
+      </c>
+      <c r="M34" s="2" t="n">
+        <v>6</v>
+      </c>
+      <c r="N34" s="2" t="n">
+        <v>10140</v>
+      </c>
+      <c r="O34" s="2" t="n">
+        <v>6</v>
+      </c>
+      <c r="P34" s="2" t="n">
+        <v>104.7</v>
+      </c>
       <c r="Q34" s="2" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="R34" s="2" t="inlineStr"/>
-      <c r="S34" s="2" t="inlineStr"/>
+      <c r="S34" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-18T22:21:26</t>
+        </is>
+      </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
@@ -2452,14 +2991,32 @@
       </c>
       <c r="K35" t="inlineStr">
         <is>
-          <t>pending</t>
-        </is>
+          <t>done</t>
+        </is>
+      </c>
+      <c r="L35" t="n">
+        <v>283</v>
+      </c>
+      <c r="M35" t="n">
+        <v>6</v>
+      </c>
+      <c r="N35" t="n">
+        <v>9735</v>
+      </c>
+      <c r="O35" t="n">
+        <v>7</v>
+      </c>
+      <c r="P35" t="n">
+        <v>103.6</v>
       </c>
       <c r="Q35" t="n">
-        <v>0</v>
-      </c>
-      <c r="R35" t="inlineStr"/>
-      <c r="S35" t="inlineStr"/>
+        <v>1</v>
+      </c>
+      <c r="S35" t="inlineStr">
+        <is>
+          <t>2026-09-18T22:23:10</t>
+        </is>
+      </c>
     </row>
     <row r="36">
       <c r="A36" s="2" t="inlineStr">
@@ -2506,19 +3063,33 @@
       </c>
       <c r="K36" s="2" t="inlineStr">
         <is>
-          <t>pending</t>
-        </is>
-      </c>
-      <c r="L36" s="2" t="n"/>
-      <c r="M36" s="2" t="n"/>
-      <c r="N36" s="2" t="n"/>
-      <c r="O36" s="2" t="n"/>
-      <c r="P36" s="2" t="n"/>
+          <t>done</t>
+        </is>
+      </c>
+      <c r="L36" s="2" t="n">
+        <v>284</v>
+      </c>
+      <c r="M36" s="2" t="n">
+        <v>6</v>
+      </c>
+      <c r="N36" s="2" t="n">
+        <v>9528</v>
+      </c>
+      <c r="O36" s="2" t="n">
+        <v>5</v>
+      </c>
+      <c r="P36" s="2" t="n">
+        <v>99.3</v>
+      </c>
       <c r="Q36" s="2" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="R36" s="2" t="inlineStr"/>
-      <c r="S36" s="2" t="inlineStr"/>
+      <c r="S36" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-18T22:24:50</t>
+        </is>
+      </c>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
@@ -2565,14 +3136,32 @@
       </c>
       <c r="K37" t="inlineStr">
         <is>
-          <t>pending</t>
-        </is>
+          <t>done</t>
+        </is>
+      </c>
+      <c r="L37" t="n">
+        <v>285</v>
+      </c>
+      <c r="M37" t="n">
+        <v>6</v>
+      </c>
+      <c r="N37" t="n">
+        <v>10165</v>
+      </c>
+      <c r="O37" t="n">
+        <v>5</v>
+      </c>
+      <c r="P37" t="n">
+        <v>95.7</v>
       </c>
       <c r="Q37" t="n">
-        <v>0</v>
-      </c>
-      <c r="R37" t="inlineStr"/>
-      <c r="S37" t="inlineStr"/>
+        <v>1</v>
+      </c>
+      <c r="S37" t="inlineStr">
+        <is>
+          <t>2026-09-18T22:26:26</t>
+        </is>
+      </c>
     </row>
     <row r="38">
       <c r="A38" s="2" t="inlineStr">
@@ -2619,19 +3208,33 @@
       </c>
       <c r="K38" s="2" t="inlineStr">
         <is>
-          <t>pending</t>
-        </is>
-      </c>
-      <c r="L38" s="2" t="n"/>
-      <c r="M38" s="2" t="n"/>
-      <c r="N38" s="2" t="n"/>
-      <c r="O38" s="2" t="n"/>
-      <c r="P38" s="2" t="n"/>
+          <t>done</t>
+        </is>
+      </c>
+      <c r="L38" s="2" t="n">
+        <v>286</v>
+      </c>
+      <c r="M38" s="2" t="n">
+        <v>7</v>
+      </c>
+      <c r="N38" s="2" t="n">
+        <v>14132</v>
+      </c>
+      <c r="O38" s="2" t="n">
+        <v>6</v>
+      </c>
+      <c r="P38" s="2" t="n">
+        <v>363.8</v>
+      </c>
       <c r="Q38" s="2" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="R38" s="2" t="inlineStr"/>
-      <c r="S38" s="2" t="inlineStr"/>
+      <c r="S38" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-18T22:32:30</t>
+        </is>
+      </c>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
@@ -2678,14 +3281,32 @@
       </c>
       <c r="K39" t="inlineStr">
         <is>
-          <t>pending</t>
-        </is>
+          <t>done</t>
+        </is>
+      </c>
+      <c r="L39" t="n">
+        <v>287</v>
+      </c>
+      <c r="M39" t="n">
+        <v>8</v>
+      </c>
+      <c r="N39" t="n">
+        <v>14659</v>
+      </c>
+      <c r="O39" t="n">
+        <v>7</v>
+      </c>
+      <c r="P39" t="n">
+        <v>140.4</v>
       </c>
       <c r="Q39" t="n">
-        <v>0</v>
-      </c>
-      <c r="R39" t="inlineStr"/>
-      <c r="S39" t="inlineStr"/>
+        <v>1</v>
+      </c>
+      <c r="S39" t="inlineStr">
+        <is>
+          <t>2026-09-18T22:34:51</t>
+        </is>
+      </c>
     </row>
     <row r="40">
       <c r="A40" s="2" t="inlineStr">
@@ -2732,19 +3353,33 @@
       </c>
       <c r="K40" s="2" t="inlineStr">
         <is>
-          <t>pending</t>
-        </is>
-      </c>
-      <c r="L40" s="2" t="n"/>
-      <c r="M40" s="2" t="n"/>
-      <c r="N40" s="2" t="n"/>
-      <c r="O40" s="2" t="n"/>
-      <c r="P40" s="2" t="n"/>
+          <t>done</t>
+        </is>
+      </c>
+      <c r="L40" s="2" t="n">
+        <v>288</v>
+      </c>
+      <c r="M40" s="2" t="n">
+        <v>9</v>
+      </c>
+      <c r="N40" s="2" t="n">
+        <v>15769</v>
+      </c>
+      <c r="O40" s="2" t="n">
+        <v>8</v>
+      </c>
+      <c r="P40" s="2" t="n">
+        <v>144.6</v>
+      </c>
       <c r="Q40" s="2" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="R40" s="2" t="inlineStr"/>
-      <c r="S40" s="2" t="inlineStr"/>
+      <c r="S40" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-18T22:37:17</t>
+        </is>
+      </c>
     </row>
     <row r="41">
       <c r="A41" t="inlineStr">
@@ -2791,14 +3426,32 @@
       </c>
       <c r="K41" t="inlineStr">
         <is>
-          <t>pending</t>
-        </is>
+          <t>done</t>
+        </is>
+      </c>
+      <c r="L41" t="n">
+        <v>289</v>
+      </c>
+      <c r="M41" t="n">
+        <v>13</v>
+      </c>
+      <c r="N41" t="n">
+        <v>20425</v>
+      </c>
+      <c r="O41" t="n">
+        <v>7</v>
+      </c>
+      <c r="P41" t="n">
+        <v>962.2</v>
       </c>
       <c r="Q41" t="n">
-        <v>0</v>
-      </c>
-      <c r="R41" t="inlineStr"/>
-      <c r="S41" t="inlineStr"/>
+        <v>1</v>
+      </c>
+      <c r="S41" t="inlineStr">
+        <is>
+          <t>2026-09-18T22:53:20</t>
+        </is>
+      </c>
     </row>
     <row r="42">
       <c r="A42" t="inlineStr">
@@ -2845,14 +3498,32 @@
       </c>
       <c r="K42" t="inlineStr">
         <is>
-          <t>pending</t>
-        </is>
+          <t>done</t>
+        </is>
+      </c>
+      <c r="L42" t="n">
+        <v>290</v>
+      </c>
+      <c r="M42" t="n">
+        <v>16</v>
+      </c>
+      <c r="N42" t="n">
+        <v>19900</v>
+      </c>
+      <c r="O42" t="n">
+        <v>13</v>
+      </c>
+      <c r="P42" t="n">
+        <v>742.4</v>
       </c>
       <c r="Q42" t="n">
-        <v>0</v>
-      </c>
-      <c r="R42" t="inlineStr"/>
-      <c r="S42" t="inlineStr"/>
+        <v>1</v>
+      </c>
+      <c r="S42" t="inlineStr">
+        <is>
+          <t>2026-09-18T23:05:43</t>
+        </is>
+      </c>
     </row>
     <row r="43">
       <c r="A43" s="2" t="inlineStr">
@@ -2899,19 +3570,33 @@
       </c>
       <c r="K43" s="2" t="inlineStr">
         <is>
-          <t>pending</t>
-        </is>
-      </c>
-      <c r="L43" s="2" t="n"/>
-      <c r="M43" s="2" t="n"/>
-      <c r="N43" s="2" t="n"/>
-      <c r="O43" s="2" t="n"/>
-      <c r="P43" s="2" t="n"/>
+          <t>done</t>
+        </is>
+      </c>
+      <c r="L43" s="2" t="n">
+        <v>291</v>
+      </c>
+      <c r="M43" s="2" t="n">
+        <v>14</v>
+      </c>
+      <c r="N43" s="2" t="n">
+        <v>17063</v>
+      </c>
+      <c r="O43" s="2" t="n">
+        <v>13</v>
+      </c>
+      <c r="P43" s="2" t="n">
+        <v>277.9</v>
+      </c>
       <c r="Q43" s="2" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="R43" s="2" t="inlineStr"/>
-      <c r="S43" s="2" t="inlineStr"/>
+      <c r="S43" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-18T23:10:22</t>
+        </is>
+      </c>
     </row>
     <row r="44">
       <c r="A44" t="inlineStr">
@@ -2958,14 +3643,32 @@
       </c>
       <c r="K44" t="inlineStr">
         <is>
-          <t>pending</t>
-        </is>
+          <t>done</t>
+        </is>
+      </c>
+      <c r="L44" t="n">
+        <v>292</v>
+      </c>
+      <c r="M44" t="n">
+        <v>14</v>
+      </c>
+      <c r="N44" t="n">
+        <v>17233</v>
+      </c>
+      <c r="O44" t="n">
+        <v>12</v>
+      </c>
+      <c r="P44" t="n">
+        <v>230.8</v>
       </c>
       <c r="Q44" t="n">
-        <v>0</v>
-      </c>
-      <c r="R44" t="inlineStr"/>
-      <c r="S44" t="inlineStr"/>
+        <v>1</v>
+      </c>
+      <c r="S44" t="inlineStr">
+        <is>
+          <t>2026-09-18T23:14:13</t>
+        </is>
+      </c>
     </row>
     <row r="45">
       <c r="A45" s="2" t="inlineStr">
@@ -3012,19 +3715,29 @@
       </c>
       <c r="K45" s="2" t="inlineStr">
         <is>
-          <t>pending</t>
+          <t>failed</t>
         </is>
       </c>
       <c r="L45" s="2" t="n"/>
       <c r="M45" s="2" t="n"/>
       <c r="N45" s="2" t="n"/>
       <c r="O45" s="2" t="n"/>
-      <c r="P45" s="2" t="n"/>
+      <c r="P45" s="2" t="n">
+        <v>107.1</v>
+      </c>
       <c r="Q45" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="R45" s="2" t="inlineStr"/>
-      <c r="S45" s="2" t="inlineStr"/>
+        <v>1</v>
+      </c>
+      <c r="R45" s="2" t="inlineStr">
+        <is>
+          <t>pdf fetch failed: 4 download attempts failed: Network error downloading PDF: Cannot connect to host ncert.nic.in:443 ssl:default [The specified network name is no longer available]; fallback also failed: HTTP 404 when fetching PDF from https://ncert.nic.in/textbook/pdf/jewe204.pdf</t>
+        </is>
+      </c>
+      <c r="S45" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-18T23:16:01</t>
+        </is>
+      </c>
     </row>
     <row r="46">
       <c r="A46" t="inlineStr">
@@ -3071,14 +3784,32 @@
       </c>
       <c r="K46" t="inlineStr">
         <is>
-          <t>pending</t>
-        </is>
+          <t>done</t>
+        </is>
+      </c>
+      <c r="L46" t="n">
+        <v>293</v>
+      </c>
+      <c r="M46" t="n">
+        <v>16</v>
+      </c>
+      <c r="N46" t="n">
+        <v>19515</v>
+      </c>
+      <c r="O46" t="n">
+        <v>15</v>
+      </c>
+      <c r="P46" t="n">
+        <v>155.9</v>
       </c>
       <c r="Q46" t="n">
-        <v>0</v>
-      </c>
-      <c r="R46" t="inlineStr"/>
-      <c r="S46" t="inlineStr"/>
+        <v>1</v>
+      </c>
+      <c r="S46" t="inlineStr">
+        <is>
+          <t>2026-09-18T23:18:37</t>
+        </is>
+      </c>
     </row>
     <row r="47">
       <c r="A47" s="2" t="inlineStr">
@@ -3125,19 +3856,33 @@
       </c>
       <c r="K47" s="2" t="inlineStr">
         <is>
-          <t>pending</t>
-        </is>
-      </c>
-      <c r="L47" s="2" t="n"/>
-      <c r="M47" s="2" t="n"/>
-      <c r="N47" s="2" t="n"/>
-      <c r="O47" s="2" t="n"/>
-      <c r="P47" s="2" t="n"/>
+          <t>done</t>
+        </is>
+      </c>
+      <c r="L47" s="2" t="n">
+        <v>294</v>
+      </c>
+      <c r="M47" s="2" t="n">
+        <v>20</v>
+      </c>
+      <c r="N47" s="2" t="n">
+        <v>21985</v>
+      </c>
+      <c r="O47" s="2" t="n">
+        <v>14</v>
+      </c>
+      <c r="P47" s="2" t="n">
+        <v>335.7</v>
+      </c>
       <c r="Q47" s="2" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="R47" s="2" t="inlineStr"/>
-      <c r="S47" s="2" t="inlineStr"/>
+      <c r="S47" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-18T23:24:15</t>
+        </is>
+      </c>
     </row>
     <row r="48">
       <c r="A48" t="inlineStr">
@@ -3184,14 +3929,32 @@
       </c>
       <c r="K48" t="inlineStr">
         <is>
-          <t>pending</t>
-        </is>
+          <t>done</t>
+        </is>
+      </c>
+      <c r="L48" t="n">
+        <v>295</v>
+      </c>
+      <c r="M48" t="n">
+        <v>16</v>
+      </c>
+      <c r="N48" t="n">
+        <v>17303</v>
+      </c>
+      <c r="O48" t="n">
+        <v>11</v>
+      </c>
+      <c r="P48" t="n">
+        <v>191.9</v>
       </c>
       <c r="Q48" t="n">
-        <v>0</v>
-      </c>
-      <c r="R48" t="inlineStr"/>
-      <c r="S48" t="inlineStr"/>
+        <v>1</v>
+      </c>
+      <c r="S48" t="inlineStr">
+        <is>
+          <t>2026-09-18T23:27:27</t>
+        </is>
+      </c>
     </row>
     <row r="49">
       <c r="A49" s="2" t="inlineStr">
@@ -3238,19 +4001,33 @@
       </c>
       <c r="K49" s="2" t="inlineStr">
         <is>
-          <t>pending</t>
-        </is>
-      </c>
-      <c r="L49" s="2" t="n"/>
-      <c r="M49" s="2" t="n"/>
-      <c r="N49" s="2" t="n"/>
-      <c r="O49" s="2" t="n"/>
-      <c r="P49" s="2" t="n"/>
+          <t>done</t>
+        </is>
+      </c>
+      <c r="L49" s="2" t="n">
+        <v>296</v>
+      </c>
+      <c r="M49" s="2" t="n">
+        <v>15</v>
+      </c>
+      <c r="N49" s="2" t="n">
+        <v>15697</v>
+      </c>
+      <c r="O49" s="2" t="n">
+        <v>11</v>
+      </c>
+      <c r="P49" s="2" t="n">
+        <v>135.9</v>
+      </c>
       <c r="Q49" s="2" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="R49" s="2" t="inlineStr"/>
-      <c r="S49" s="2" t="inlineStr"/>
+      <c r="S49" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-18T23:29:43</t>
+        </is>
+      </c>
     </row>
     <row r="50">
       <c r="A50" t="inlineStr">
@@ -3297,14 +4074,25 @@
       </c>
       <c r="K50" t="inlineStr">
         <is>
-          <t>pending</t>
-        </is>
+          <t>failed</t>
+        </is>
+      </c>
+      <c r="P50" t="n">
+        <v>107.4</v>
       </c>
       <c r="Q50" t="n">
-        <v>0</v>
-      </c>
-      <c r="R50" t="inlineStr"/>
-      <c r="S50" t="inlineStr"/>
+        <v>1</v>
+      </c>
+      <c r="R50" t="inlineStr">
+        <is>
+          <t>pdf fetch failed: 4 download attempts failed: HTTP 404 when fetching PDF from https://ncert.nic.in/textbook/pdf/jewe209.pdf</t>
+        </is>
+      </c>
+      <c r="S50" t="inlineStr">
+        <is>
+          <t>2026-09-18T23:31:31</t>
+        </is>
+      </c>
     </row>
     <row r="51">
       <c r="A51" t="inlineStr">
@@ -3351,14 +4139,32 @@
       </c>
       <c r="K51" t="inlineStr">
         <is>
-          <t>pending</t>
-        </is>
+          <t>done</t>
+        </is>
+      </c>
+      <c r="L51" t="n">
+        <v>297</v>
+      </c>
+      <c r="M51" t="n">
+        <v>9</v>
+      </c>
+      <c r="N51" t="n">
+        <v>6368</v>
+      </c>
+      <c r="O51" t="n">
+        <v>3</v>
+      </c>
+      <c r="P51" t="n">
+        <v>68.5</v>
       </c>
       <c r="Q51" t="n">
-        <v>0</v>
-      </c>
-      <c r="R51" t="inlineStr"/>
-      <c r="S51" t="inlineStr"/>
+        <v>1</v>
+      </c>
+      <c r="S51" t="inlineStr">
+        <is>
+          <t>2026-09-18T23:32:40</t>
+        </is>
+      </c>
     </row>
     <row r="52">
       <c r="A52" s="2" t="inlineStr">
@@ -3405,19 +4211,33 @@
       </c>
       <c r="K52" s="2" t="inlineStr">
         <is>
-          <t>pending</t>
-        </is>
-      </c>
-      <c r="L52" s="2" t="n"/>
-      <c r="M52" s="2" t="n"/>
-      <c r="N52" s="2" t="n"/>
-      <c r="O52" s="2" t="n"/>
-      <c r="P52" s="2" t="n"/>
+          <t>done</t>
+        </is>
+      </c>
+      <c r="L52" s="2" t="n">
+        <v>298</v>
+      </c>
+      <c r="M52" s="2" t="n">
+        <v>7</v>
+      </c>
+      <c r="N52" s="2" t="n">
+        <v>6913</v>
+      </c>
+      <c r="O52" s="2" t="n">
+        <v>3</v>
+      </c>
+      <c r="P52" s="2" t="n">
+        <v>77.8</v>
+      </c>
       <c r="Q52" s="2" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="R52" s="2" t="inlineStr"/>
-      <c r="S52" s="2" t="inlineStr"/>
+      <c r="S52" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-18T23:33:58</t>
+        </is>
+      </c>
     </row>
     <row r="53">
       <c r="A53" t="inlineStr">
@@ -3464,14 +4284,32 @@
       </c>
       <c r="K53" t="inlineStr">
         <is>
-          <t>pending</t>
-        </is>
+          <t>done</t>
+        </is>
+      </c>
+      <c r="L53" t="n">
+        <v>299</v>
+      </c>
+      <c r="M53" t="n">
+        <v>5</v>
+      </c>
+      <c r="N53" t="n">
+        <v>4859</v>
+      </c>
+      <c r="O53" t="n">
+        <v>2</v>
+      </c>
+      <c r="P53" t="n">
+        <v>45.7</v>
       </c>
       <c r="Q53" t="n">
-        <v>0</v>
-      </c>
-      <c r="R53" t="inlineStr"/>
-      <c r="S53" t="inlineStr"/>
+        <v>1</v>
+      </c>
+      <c r="S53" t="inlineStr">
+        <is>
+          <t>2026-09-18T23:34:44</t>
+        </is>
+      </c>
     </row>
     <row r="54">
       <c r="A54" s="2" t="inlineStr">
@@ -3518,19 +4356,33 @@
       </c>
       <c r="K54" s="2" t="inlineStr">
         <is>
-          <t>pending</t>
-        </is>
-      </c>
-      <c r="L54" s="2" t="n"/>
-      <c r="M54" s="2" t="n"/>
-      <c r="N54" s="2" t="n"/>
-      <c r="O54" s="2" t="n"/>
-      <c r="P54" s="2" t="n"/>
+          <t>done</t>
+        </is>
+      </c>
+      <c r="L54" s="2" t="n">
+        <v>300</v>
+      </c>
+      <c r="M54" s="2" t="n">
+        <v>6</v>
+      </c>
+      <c r="N54" s="2" t="n">
+        <v>4451</v>
+      </c>
+      <c r="O54" s="2" t="n">
+        <v>3</v>
+      </c>
+      <c r="P54" s="2" t="n">
+        <v>43.3</v>
+      </c>
       <c r="Q54" s="2" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="R54" s="2" t="inlineStr"/>
-      <c r="S54" s="2" t="inlineStr"/>
+      <c r="S54" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-18T23:35:28</t>
+        </is>
+      </c>
     </row>
     <row r="55">
       <c r="A55" t="inlineStr">
@@ -3577,14 +4429,32 @@
       </c>
       <c r="K55" t="inlineStr">
         <is>
-          <t>pending</t>
-        </is>
+          <t>done</t>
+        </is>
+      </c>
+      <c r="L55" t="n">
+        <v>301</v>
+      </c>
+      <c r="M55" t="n">
+        <v>7</v>
+      </c>
+      <c r="N55" t="n">
+        <v>5932</v>
+      </c>
+      <c r="O55" t="n">
+        <v>4</v>
+      </c>
+      <c r="P55" t="n">
+        <v>59.8</v>
       </c>
       <c r="Q55" t="n">
-        <v>0</v>
-      </c>
-      <c r="R55" t="inlineStr"/>
-      <c r="S55" t="inlineStr"/>
+        <v>1</v>
+      </c>
+      <c r="S55" t="inlineStr">
+        <is>
+          <t>2026-09-18T23:36:29</t>
+        </is>
+      </c>
     </row>
     <row r="56">
       <c r="A56" s="2" t="inlineStr">
@@ -3631,19 +4501,33 @@
       </c>
       <c r="K56" s="2" t="inlineStr">
         <is>
-          <t>pending</t>
-        </is>
-      </c>
-      <c r="L56" s="2" t="n"/>
-      <c r="M56" s="2" t="n"/>
-      <c r="N56" s="2" t="n"/>
-      <c r="O56" s="2" t="n"/>
-      <c r="P56" s="2" t="n"/>
+          <t>done</t>
+        </is>
+      </c>
+      <c r="L56" s="2" t="n">
+        <v>302</v>
+      </c>
+      <c r="M56" s="2" t="n">
+        <v>8</v>
+      </c>
+      <c r="N56" s="2" t="n">
+        <v>6047</v>
+      </c>
+      <c r="O56" s="2" t="n">
+        <v>5</v>
+      </c>
+      <c r="P56" s="2" t="n">
+        <v>63.3</v>
+      </c>
       <c r="Q56" s="2" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="R56" s="2" t="inlineStr"/>
-      <c r="S56" s="2" t="inlineStr"/>
+      <c r="S56" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-18T23:37:33</t>
+        </is>
+      </c>
     </row>
     <row r="57">
       <c r="A57" t="inlineStr">
@@ -3690,14 +4574,32 @@
       </c>
       <c r="K57" t="inlineStr">
         <is>
-          <t>pending</t>
-        </is>
+          <t>done</t>
+        </is>
+      </c>
+      <c r="L57" t="n">
+        <v>303</v>
+      </c>
+      <c r="M57" t="n">
+        <v>9</v>
+      </c>
+      <c r="N57" t="n">
+        <v>13770</v>
+      </c>
+      <c r="O57" t="n">
+        <v>3</v>
+      </c>
+      <c r="P57" t="n">
+        <v>139</v>
       </c>
       <c r="Q57" t="n">
-        <v>0</v>
-      </c>
-      <c r="R57" t="inlineStr"/>
-      <c r="S57" t="inlineStr"/>
+        <v>1</v>
+      </c>
+      <c r="S57" t="inlineStr">
+        <is>
+          <t>2026-09-18T23:39:52</t>
+        </is>
+      </c>
     </row>
     <row r="58">
       <c r="A58" s="2" t="inlineStr">
@@ -3744,19 +4646,33 @@
       </c>
       <c r="K58" s="2" t="inlineStr">
         <is>
-          <t>pending</t>
-        </is>
-      </c>
-      <c r="L58" s="2" t="n"/>
-      <c r="M58" s="2" t="n"/>
-      <c r="N58" s="2" t="n"/>
-      <c r="O58" s="2" t="n"/>
-      <c r="P58" s="2" t="n"/>
+          <t>done</t>
+        </is>
+      </c>
+      <c r="L58" s="2" t="n">
+        <v>304</v>
+      </c>
+      <c r="M58" s="2" t="n">
+        <v>9</v>
+      </c>
+      <c r="N58" s="2" t="n">
+        <v>11511</v>
+      </c>
+      <c r="O58" s="2" t="n">
+        <v>4</v>
+      </c>
+      <c r="P58" s="2" t="n">
+        <v>94.59999999999999</v>
+      </c>
       <c r="Q58" s="2" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="R58" s="2" t="inlineStr"/>
-      <c r="S58" s="2" t="inlineStr"/>
+      <c r="S58" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-18T23:41:27</t>
+        </is>
+      </c>
     </row>
     <row r="59">
       <c r="A59" t="inlineStr">
@@ -3803,14 +4719,32 @@
       </c>
       <c r="K59" t="inlineStr">
         <is>
-          <t>pending</t>
-        </is>
+          <t>done</t>
+        </is>
+      </c>
+      <c r="L59" t="n">
+        <v>305</v>
+      </c>
+      <c r="M59" t="n">
+        <v>6</v>
+      </c>
+      <c r="N59" t="n">
+        <v>7408</v>
+      </c>
+      <c r="O59" t="n">
+        <v>3</v>
+      </c>
+      <c r="P59" t="n">
+        <v>69.5</v>
       </c>
       <c r="Q59" t="n">
-        <v>0</v>
-      </c>
-      <c r="R59" t="inlineStr"/>
-      <c r="S59" t="inlineStr"/>
+        <v>1</v>
+      </c>
+      <c r="S59" t="inlineStr">
+        <is>
+          <t>2026-09-18T23:42:37</t>
+        </is>
+      </c>
     </row>
     <row r="60">
       <c r="A60" s="2" t="inlineStr">
@@ -3857,19 +4791,33 @@
       </c>
       <c r="K60" s="2" t="inlineStr">
         <is>
-          <t>pending</t>
-        </is>
-      </c>
-      <c r="L60" s="2" t="n"/>
-      <c r="M60" s="2" t="n"/>
-      <c r="N60" s="2" t="n"/>
-      <c r="O60" s="2" t="n"/>
-      <c r="P60" s="2" t="n"/>
+          <t>done</t>
+        </is>
+      </c>
+      <c r="L60" s="2" t="n">
+        <v>306</v>
+      </c>
+      <c r="M60" s="2" t="n">
+        <v>12</v>
+      </c>
+      <c r="N60" s="2" t="n">
+        <v>17944</v>
+      </c>
+      <c r="O60" s="2" t="n">
+        <v>5</v>
+      </c>
+      <c r="P60" s="2" t="n">
+        <v>198.8</v>
+      </c>
       <c r="Q60" s="2" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="R60" s="2" t="inlineStr"/>
-      <c r="S60" s="2" t="inlineStr"/>
+      <c r="S60" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-18T23:45:57</t>
+        </is>
+      </c>
     </row>
     <row r="61">
       <c r="A61" t="inlineStr">
@@ -3916,14 +4864,32 @@
       </c>
       <c r="K61" t="inlineStr">
         <is>
-          <t>pending</t>
-        </is>
+          <t>done</t>
+        </is>
+      </c>
+      <c r="L61" t="n">
+        <v>307</v>
+      </c>
+      <c r="M61" t="n">
+        <v>12</v>
+      </c>
+      <c r="N61" t="n">
+        <v>16536</v>
+      </c>
+      <c r="O61" t="n">
+        <v>8</v>
+      </c>
+      <c r="P61" t="n">
+        <v>194.8</v>
       </c>
       <c r="Q61" t="n">
-        <v>0</v>
-      </c>
-      <c r="R61" t="inlineStr"/>
-      <c r="S61" t="inlineStr"/>
+        <v>1</v>
+      </c>
+      <c r="S61" t="inlineStr">
+        <is>
+          <t>2026-09-18T23:49:12</t>
+        </is>
+      </c>
     </row>
     <row r="62">
       <c r="A62" s="2" t="inlineStr">
@@ -3970,19 +4936,33 @@
       </c>
       <c r="K62" s="2" t="inlineStr">
         <is>
-          <t>pending</t>
-        </is>
-      </c>
-      <c r="L62" s="2" t="n"/>
-      <c r="M62" s="2" t="n"/>
-      <c r="N62" s="2" t="n"/>
-      <c r="O62" s="2" t="n"/>
-      <c r="P62" s="2" t="n"/>
+          <t>done</t>
+        </is>
+      </c>
+      <c r="L62" s="2" t="n">
+        <v>308</v>
+      </c>
+      <c r="M62" s="2" t="n">
+        <v>8</v>
+      </c>
+      <c r="N62" s="2" t="n">
+        <v>7959</v>
+      </c>
+      <c r="O62" s="2" t="n">
+        <v>5</v>
+      </c>
+      <c r="P62" s="2" t="n">
+        <v>127.5</v>
+      </c>
       <c r="Q62" s="2" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="R62" s="2" t="inlineStr"/>
-      <c r="S62" s="2" t="inlineStr"/>
+      <c r="S62" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-18T23:51:20</t>
+        </is>
+      </c>
     </row>
     <row r="63">
       <c r="A63" t="inlineStr">
@@ -4029,14 +5009,32 @@
       </c>
       <c r="K63" t="inlineStr">
         <is>
-          <t>pending</t>
-        </is>
+          <t>done</t>
+        </is>
+      </c>
+      <c r="L63" t="n">
+        <v>309</v>
+      </c>
+      <c r="M63" t="n">
+        <v>6</v>
+      </c>
+      <c r="N63" t="n">
+        <v>3792</v>
+      </c>
+      <c r="O63" t="n">
+        <v>2</v>
+      </c>
+      <c r="P63" t="n">
+        <v>55.9</v>
       </c>
       <c r="Q63" t="n">
-        <v>0</v>
-      </c>
-      <c r="R63" t="inlineStr"/>
-      <c r="S63" t="inlineStr"/>
+        <v>1</v>
+      </c>
+      <c r="S63" t="inlineStr">
+        <is>
+          <t>2026-09-18T23:52:19</t>
+        </is>
+      </c>
     </row>
     <row r="64">
       <c r="A64" s="2" t="inlineStr">
@@ -4083,19 +5081,33 @@
       </c>
       <c r="K64" s="2" t="inlineStr">
         <is>
-          <t>pending</t>
-        </is>
-      </c>
-      <c r="L64" s="2" t="n"/>
-      <c r="M64" s="2" t="n"/>
-      <c r="N64" s="2" t="n"/>
-      <c r="O64" s="2" t="n"/>
-      <c r="P64" s="2" t="n"/>
+          <t>done</t>
+        </is>
+      </c>
+      <c r="L64" s="2" t="n">
+        <v>310</v>
+      </c>
+      <c r="M64" s="2" t="n">
+        <v>5</v>
+      </c>
+      <c r="N64" s="2" t="n">
+        <v>3741</v>
+      </c>
+      <c r="O64" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="P64" s="2" t="n">
+        <v>56.7</v>
+      </c>
       <c r="Q64" s="2" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="R64" s="2" t="inlineStr"/>
-      <c r="S64" s="2" t="inlineStr"/>
+      <c r="S64" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-18T23:53:16</t>
+        </is>
+      </c>
     </row>
     <row r="65">
       <c r="A65" t="inlineStr">
@@ -4142,14 +5154,32 @@
       </c>
       <c r="K65" t="inlineStr">
         <is>
-          <t>pending</t>
-        </is>
+          <t>done</t>
+        </is>
+      </c>
+      <c r="L65" t="n">
+        <v>311</v>
+      </c>
+      <c r="M65" t="n">
+        <v>7</v>
+      </c>
+      <c r="N65" t="n">
+        <v>5129</v>
+      </c>
+      <c r="O65" t="n">
+        <v>1</v>
+      </c>
+      <c r="P65" t="n">
+        <v>69.09999999999999</v>
       </c>
       <c r="Q65" t="n">
-        <v>0</v>
-      </c>
-      <c r="R65" t="inlineStr"/>
-      <c r="S65" t="inlineStr"/>
+        <v>1</v>
+      </c>
+      <c r="S65" t="inlineStr">
+        <is>
+          <t>2026-09-18T23:54:25</t>
+        </is>
+      </c>
     </row>
     <row r="66">
       <c r="A66" s="2" t="inlineStr">
@@ -4196,19 +5226,33 @@
       </c>
       <c r="K66" s="2" t="inlineStr">
         <is>
-          <t>pending</t>
-        </is>
-      </c>
-      <c r="L66" s="2" t="n"/>
-      <c r="M66" s="2" t="n"/>
-      <c r="N66" s="2" t="n"/>
-      <c r="O66" s="2" t="n"/>
-      <c r="P66" s="2" t="n"/>
+          <t>done</t>
+        </is>
+      </c>
+      <c r="L66" s="2" t="n">
+        <v>312</v>
+      </c>
+      <c r="M66" s="2" t="n">
+        <v>6</v>
+      </c>
+      <c r="N66" s="2" t="n">
+        <v>4051</v>
+      </c>
+      <c r="O66" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="P66" s="2" t="n">
+        <v>59.3</v>
+      </c>
       <c r="Q66" s="2" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="R66" s="2" t="inlineStr"/>
-      <c r="S66" s="2" t="inlineStr"/>
+      <c r="S66" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-18T23:55:25</t>
+        </is>
+      </c>
     </row>
     <row r="67">
       <c r="A67" t="inlineStr">
@@ -4255,14 +5299,32 @@
       </c>
       <c r="K67" t="inlineStr">
         <is>
-          <t>pending</t>
-        </is>
+          <t>done</t>
+        </is>
+      </c>
+      <c r="L67" t="n">
+        <v>313</v>
+      </c>
+      <c r="M67" t="n">
+        <v>5</v>
+      </c>
+      <c r="N67" t="n">
+        <v>3675</v>
+      </c>
+      <c r="O67" t="n">
+        <v>1</v>
+      </c>
+      <c r="P67" t="n">
+        <v>43.7</v>
       </c>
       <c r="Q67" t="n">
-        <v>0</v>
-      </c>
-      <c r="R67" t="inlineStr"/>
-      <c r="S67" t="inlineStr"/>
+        <v>1</v>
+      </c>
+      <c r="S67" t="inlineStr">
+        <is>
+          <t>2026-09-18T23:56:09</t>
+        </is>
+      </c>
     </row>
     <row r="68">
       <c r="A68" s="2" t="inlineStr">
@@ -4309,19 +5371,33 @@
       </c>
       <c r="K68" s="2" t="inlineStr">
         <is>
-          <t>pending</t>
-        </is>
-      </c>
-      <c r="L68" s="2" t="n"/>
-      <c r="M68" s="2" t="n"/>
-      <c r="N68" s="2" t="n"/>
-      <c r="O68" s="2" t="n"/>
-      <c r="P68" s="2" t="n"/>
+          <t>done</t>
+        </is>
+      </c>
+      <c r="L68" s="2" t="n">
+        <v>314</v>
+      </c>
+      <c r="M68" s="2" t="n">
+        <v>5</v>
+      </c>
+      <c r="N68" s="2" t="n">
+        <v>4229</v>
+      </c>
+      <c r="O68" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="P68" s="2" t="n">
+        <v>43.9</v>
+      </c>
       <c r="Q68" s="2" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="R68" s="2" t="inlineStr"/>
-      <c r="S68" s="2" t="inlineStr"/>
+      <c r="S68" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-18T23:56:54</t>
+        </is>
+      </c>
     </row>
     <row r="69">
       <c r="A69" t="inlineStr">
@@ -4368,14 +5444,32 @@
       </c>
       <c r="K69" t="inlineStr">
         <is>
-          <t>pending</t>
-        </is>
+          <t>done</t>
+        </is>
+      </c>
+      <c r="L69" t="n">
+        <v>315</v>
+      </c>
+      <c r="M69" t="n">
+        <v>5</v>
+      </c>
+      <c r="N69" t="n">
+        <v>4209</v>
+      </c>
+      <c r="O69" t="n">
+        <v>0</v>
+      </c>
+      <c r="P69" t="n">
+        <v>47.1</v>
       </c>
       <c r="Q69" t="n">
-        <v>0</v>
-      </c>
-      <c r="R69" t="inlineStr"/>
-      <c r="S69" t="inlineStr"/>
+        <v>1</v>
+      </c>
+      <c r="S69" t="inlineStr">
+        <is>
+          <t>2026-09-18T23:57:41</t>
+        </is>
+      </c>
     </row>
     <row r="70">
       <c r="A70" s="2" t="inlineStr">
@@ -4422,19 +5516,33 @@
       </c>
       <c r="K70" s="2" t="inlineStr">
         <is>
-          <t>pending</t>
-        </is>
-      </c>
-      <c r="L70" s="2" t="n"/>
-      <c r="M70" s="2" t="n"/>
-      <c r="N70" s="2" t="n"/>
-      <c r="O70" s="2" t="n"/>
-      <c r="P70" s="2" t="n"/>
+          <t>done</t>
+        </is>
+      </c>
+      <c r="L70" s="2" t="n">
+        <v>316</v>
+      </c>
+      <c r="M70" s="2" t="n">
+        <v>16</v>
+      </c>
+      <c r="N70" s="2" t="n">
+        <v>22821</v>
+      </c>
+      <c r="O70" s="2" t="n">
+        <v>5</v>
+      </c>
+      <c r="P70" s="2" t="n">
+        <v>181.5</v>
+      </c>
       <c r="Q70" s="2" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="R70" s="2" t="inlineStr"/>
-      <c r="S70" s="2" t="inlineStr"/>
+      <c r="S70" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-19T00:00:43</t>
+        </is>
+      </c>
     </row>
     <row r="71">
       <c r="A71" t="inlineStr">
@@ -4481,14 +5589,32 @@
       </c>
       <c r="K71" t="inlineStr">
         <is>
-          <t>pending</t>
-        </is>
+          <t>done</t>
+        </is>
+      </c>
+      <c r="L71" t="n">
+        <v>317</v>
+      </c>
+      <c r="M71" t="n">
+        <v>9</v>
+      </c>
+      <c r="N71" t="n">
+        <v>13104</v>
+      </c>
+      <c r="O71" t="n">
+        <v>2</v>
+      </c>
+      <c r="P71" t="n">
+        <v>119.5</v>
       </c>
       <c r="Q71" t="n">
-        <v>0</v>
-      </c>
-      <c r="R71" t="inlineStr"/>
-      <c r="S71" t="inlineStr"/>
+        <v>1</v>
+      </c>
+      <c r="S71" t="inlineStr">
+        <is>
+          <t>2026-09-19T00:02:43</t>
+        </is>
+      </c>
     </row>
     <row r="72">
       <c r="A72" s="2" t="inlineStr">
@@ -4535,19 +5661,33 @@
       </c>
       <c r="K72" s="2" t="inlineStr">
         <is>
-          <t>pending</t>
-        </is>
-      </c>
-      <c r="L72" s="2" t="n"/>
-      <c r="M72" s="2" t="n"/>
-      <c r="N72" s="2" t="n"/>
-      <c r="O72" s="2" t="n"/>
-      <c r="P72" s="2" t="n"/>
+          <t>done</t>
+        </is>
+      </c>
+      <c r="L72" s="2" t="n">
+        <v>318</v>
+      </c>
+      <c r="M72" s="2" t="n">
+        <v>12</v>
+      </c>
+      <c r="N72" s="2" t="n">
+        <v>16607</v>
+      </c>
+      <c r="O72" s="2" t="n">
+        <v>4</v>
+      </c>
+      <c r="P72" s="2" t="n">
+        <v>128.8</v>
+      </c>
       <c r="Q72" s="2" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="R72" s="2" t="inlineStr"/>
-      <c r="S72" s="2" t="inlineStr"/>
+      <c r="S72" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-19T00:04:53</t>
+        </is>
+      </c>
     </row>
     <row r="73">
       <c r="A73" t="inlineStr">
@@ -4594,14 +5734,32 @@
       </c>
       <c r="K73" t="inlineStr">
         <is>
-          <t>pending</t>
-        </is>
+          <t>done</t>
+        </is>
+      </c>
+      <c r="L73" t="n">
+        <v>319</v>
+      </c>
+      <c r="M73" t="n">
+        <v>10</v>
+      </c>
+      <c r="N73" t="n">
+        <v>13144</v>
+      </c>
+      <c r="O73" t="n">
+        <v>2</v>
+      </c>
+      <c r="P73" t="n">
+        <v>120.8</v>
       </c>
       <c r="Q73" t="n">
-        <v>0</v>
-      </c>
-      <c r="R73" t="inlineStr"/>
-      <c r="S73" t="inlineStr"/>
+        <v>1</v>
+      </c>
+      <c r="S73" t="inlineStr">
+        <is>
+          <t>2026-09-19T00:06:55</t>
+        </is>
+      </c>
     </row>
     <row r="74">
       <c r="A74" s="2" t="inlineStr">
@@ -4648,19 +5806,33 @@
       </c>
       <c r="K74" s="2" t="inlineStr">
         <is>
-          <t>pending</t>
-        </is>
-      </c>
-      <c r="L74" s="2" t="n"/>
-      <c r="M74" s="2" t="n"/>
-      <c r="N74" s="2" t="n"/>
-      <c r="O74" s="2" t="n"/>
-      <c r="P74" s="2" t="n"/>
+          <t>done</t>
+        </is>
+      </c>
+      <c r="L74" s="2" t="n">
+        <v>320</v>
+      </c>
+      <c r="M74" s="2" t="n">
+        <v>8</v>
+      </c>
+      <c r="N74" s="2" t="n">
+        <v>10221</v>
+      </c>
+      <c r="O74" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="P74" s="2" t="n">
+        <v>93.7</v>
+      </c>
       <c r="Q74" s="2" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="R74" s="2" t="inlineStr"/>
-      <c r="S74" s="2" t="inlineStr"/>
+      <c r="S74" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-19T00:08:29</t>
+        </is>
+      </c>
     </row>
     <row r="75">
       <c r="A75" t="inlineStr">
@@ -4707,14 +5879,32 @@
       </c>
       <c r="K75" t="inlineStr">
         <is>
-          <t>pending</t>
-        </is>
+          <t>done</t>
+        </is>
+      </c>
+      <c r="L75" t="n">
+        <v>321</v>
+      </c>
+      <c r="M75" t="n">
+        <v>10</v>
+      </c>
+      <c r="N75" t="n">
+        <v>10099</v>
+      </c>
+      <c r="O75" t="n">
+        <v>3</v>
+      </c>
+      <c r="P75" t="n">
+        <v>89.8</v>
       </c>
       <c r="Q75" t="n">
-        <v>0</v>
-      </c>
-      <c r="R75" t="inlineStr"/>
-      <c r="S75" t="inlineStr"/>
+        <v>1</v>
+      </c>
+      <c r="S75" t="inlineStr">
+        <is>
+          <t>2026-09-19T00:09:59</t>
+        </is>
+      </c>
     </row>
     <row r="76">
       <c r="A76" s="2" t="inlineStr">
@@ -4761,19 +5951,33 @@
       </c>
       <c r="K76" s="2" t="inlineStr">
         <is>
-          <t>pending</t>
-        </is>
-      </c>
-      <c r="L76" s="2" t="n"/>
-      <c r="M76" s="2" t="n"/>
-      <c r="N76" s="2" t="n"/>
-      <c r="O76" s="2" t="n"/>
-      <c r="P76" s="2" t="n"/>
+          <t>done</t>
+        </is>
+      </c>
+      <c r="L76" s="2" t="n">
+        <v>322</v>
+      </c>
+      <c r="M76" s="2" t="n">
+        <v>10</v>
+      </c>
+      <c r="N76" s="2" t="n">
+        <v>9752</v>
+      </c>
+      <c r="O76" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="P76" s="2" t="n">
+        <v>130</v>
+      </c>
       <c r="Q76" s="2" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="R76" s="2" t="inlineStr"/>
-      <c r="S76" s="2" t="inlineStr"/>
+      <c r="S76" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-19T00:12:10</t>
+        </is>
+      </c>
     </row>
     <row r="77">
       <c r="A77" t="inlineStr">
@@ -4820,14 +6024,32 @@
       </c>
       <c r="K77" t="inlineStr">
         <is>
-          <t>pending</t>
-        </is>
+          <t>done</t>
+        </is>
+      </c>
+      <c r="L77" t="n">
+        <v>323</v>
+      </c>
+      <c r="M77" t="n">
+        <v>10</v>
+      </c>
+      <c r="N77" t="n">
+        <v>23984</v>
+      </c>
+      <c r="O77" t="n">
+        <v>7</v>
+      </c>
+      <c r="P77" t="n">
+        <v>120.4</v>
       </c>
       <c r="Q77" t="n">
-        <v>0</v>
-      </c>
-      <c r="R77" t="inlineStr"/>
-      <c r="S77" t="inlineStr"/>
+        <v>1</v>
+      </c>
+      <c r="S77" t="inlineStr">
+        <is>
+          <t>2026-09-19T00:14:11</t>
+        </is>
+      </c>
     </row>
     <row r="78">
       <c r="A78" s="2" t="inlineStr">
@@ -4874,19 +6096,33 @@
       </c>
       <c r="K78" s="2" t="inlineStr">
         <is>
-          <t>pending</t>
-        </is>
-      </c>
-      <c r="L78" s="2" t="n"/>
-      <c r="M78" s="2" t="n"/>
-      <c r="N78" s="2" t="n"/>
-      <c r="O78" s="2" t="n"/>
-      <c r="P78" s="2" t="n"/>
+          <t>done</t>
+        </is>
+      </c>
+      <c r="L78" s="2" t="n">
+        <v>324</v>
+      </c>
+      <c r="M78" s="2" t="n">
+        <v>12</v>
+      </c>
+      <c r="N78" s="2" t="n">
+        <v>22548</v>
+      </c>
+      <c r="O78" s="2" t="n">
+        <v>17</v>
+      </c>
+      <c r="P78" s="2" t="n">
+        <v>727</v>
+      </c>
       <c r="Q78" s="2" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="R78" s="2" t="inlineStr"/>
-      <c r="S78" s="2" t="inlineStr"/>
+      <c r="S78" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-19T00:26:19</t>
+        </is>
+      </c>
     </row>
     <row r="79">
       <c r="A79" t="inlineStr">
@@ -4933,14 +6169,32 @@
       </c>
       <c r="K79" t="inlineStr">
         <is>
-          <t>pending</t>
-        </is>
+          <t>done</t>
+        </is>
+      </c>
+      <c r="L79" t="n">
+        <v>325</v>
+      </c>
+      <c r="M79" t="n">
+        <v>12</v>
+      </c>
+      <c r="N79" t="n">
+        <v>23332</v>
+      </c>
+      <c r="O79" t="n">
+        <v>9</v>
+      </c>
+      <c r="P79" t="n">
+        <v>417.6</v>
       </c>
       <c r="Q79" t="n">
-        <v>0</v>
-      </c>
-      <c r="R79" t="inlineStr"/>
-      <c r="S79" t="inlineStr"/>
+        <v>1</v>
+      </c>
+      <c r="S79" t="inlineStr">
+        <is>
+          <t>2026-09-19T00:33:21</t>
+        </is>
+      </c>
     </row>
     <row r="80">
       <c r="A80" s="2" t="inlineStr">
@@ -4987,19 +6241,33 @@
       </c>
       <c r="K80" s="2" t="inlineStr">
         <is>
-          <t>pending</t>
-        </is>
-      </c>
-      <c r="L80" s="2" t="n"/>
-      <c r="M80" s="2" t="n"/>
-      <c r="N80" s="2" t="n"/>
-      <c r="O80" s="2" t="n"/>
-      <c r="P80" s="2" t="n"/>
+          <t>done</t>
+        </is>
+      </c>
+      <c r="L80" s="2" t="n">
+        <v>326</v>
+      </c>
+      <c r="M80" s="2" t="n">
+        <v>17</v>
+      </c>
+      <c r="N80" s="2" t="n">
+        <v>28304</v>
+      </c>
+      <c r="O80" s="2" t="n">
+        <v>26</v>
+      </c>
+      <c r="P80" s="2" t="n">
+        <v>1074</v>
+      </c>
       <c r="Q80" s="2" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="R80" s="2" t="inlineStr"/>
-      <c r="S80" s="2" t="inlineStr"/>
+      <c r="S80" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-19T00:51:21</t>
+        </is>
+      </c>
     </row>
     <row r="81">
       <c r="A81" t="inlineStr">
@@ -5046,14 +6314,32 @@
       </c>
       <c r="K81" t="inlineStr">
         <is>
-          <t>pending</t>
-        </is>
+          <t>done</t>
+        </is>
+      </c>
+      <c r="L81" t="n">
+        <v>327</v>
+      </c>
+      <c r="M81" t="n">
+        <v>25</v>
+      </c>
+      <c r="N81" t="n">
+        <v>43876</v>
+      </c>
+      <c r="O81" t="n">
+        <v>20</v>
+      </c>
+      <c r="P81" t="n">
+        <v>323.4</v>
       </c>
       <c r="Q81" t="n">
-        <v>0</v>
-      </c>
-      <c r="R81" t="inlineStr"/>
-      <c r="S81" t="inlineStr"/>
+        <v>1</v>
+      </c>
+      <c r="S81" t="inlineStr">
+        <is>
+          <t>2026-09-19T00:56:45</t>
+        </is>
+      </c>
     </row>
     <row r="82">
       <c r="A82" s="2" t="inlineStr">
@@ -5100,19 +6386,29 @@
       </c>
       <c r="K82" s="2" t="inlineStr">
         <is>
-          <t>pending</t>
+          <t>failed</t>
         </is>
       </c>
       <c r="L82" s="2" t="n"/>
       <c r="M82" s="2" t="n"/>
       <c r="N82" s="2" t="n"/>
       <c r="O82" s="2" t="n"/>
-      <c r="P82" s="2" t="n"/>
+      <c r="P82" s="2" t="n">
+        <v>106.7</v>
+      </c>
       <c r="Q82" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="R82" s="2" t="inlineStr"/>
-      <c r="S82" s="2" t="inlineStr"/>
+        <v>1</v>
+      </c>
+      <c r="R82" s="2" t="inlineStr">
+        <is>
+          <t>pdf fetch failed: 4 download attempts failed: Network error downloading PDF: Cannot connect to host ncert.nic.in:443 ssl:default [The specified network name is no longer available]; fallback also failed: HTTP 404 when fetching PDF from https://ncert.nic.in/textbook/pdf/jehp106.pdf</t>
+        </is>
+      </c>
+      <c r="S82" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-19T00:58:32</t>
+        </is>
+      </c>
     </row>
     <row r="83">
       <c r="A83" t="inlineStr">
@@ -5159,14 +6455,32 @@
       </c>
       <c r="K83" t="inlineStr">
         <is>
-          <t>pending</t>
-        </is>
+          <t>done</t>
+        </is>
+      </c>
+      <c r="L83" t="n">
+        <v>328</v>
+      </c>
+      <c r="M83" t="n">
+        <v>22</v>
+      </c>
+      <c r="N83" t="n">
+        <v>40713</v>
+      </c>
+      <c r="O83" t="n">
+        <v>20</v>
+      </c>
+      <c r="P83" t="n">
+        <v>1011.8</v>
       </c>
       <c r="Q83" t="n">
-        <v>0</v>
-      </c>
-      <c r="R83" t="inlineStr"/>
-      <c r="S83" t="inlineStr"/>
+        <v>1</v>
+      </c>
+      <c r="S83" t="inlineStr">
+        <is>
+          <t>2026-09-19T01:15:25</t>
+        </is>
+      </c>
     </row>
     <row r="84">
       <c r="A84" s="2" t="inlineStr">
@@ -5213,19 +6527,29 @@
       </c>
       <c r="K84" s="2" t="inlineStr">
         <is>
-          <t>pending</t>
+          <t>failed</t>
         </is>
       </c>
       <c r="L84" s="2" t="n"/>
       <c r="M84" s="2" t="n"/>
       <c r="N84" s="2" t="n"/>
       <c r="O84" s="2" t="n"/>
-      <c r="P84" s="2" t="n"/>
+      <c r="P84" s="2" t="n">
+        <v>106.7</v>
+      </c>
       <c r="Q84" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="R84" s="2" t="inlineStr"/>
-      <c r="S84" s="2" t="inlineStr"/>
+        <v>1</v>
+      </c>
+      <c r="R84" s="2" t="inlineStr">
+        <is>
+          <t>pdf fetch failed: 4 download attempts failed: HTTP 404 when fetching PDF from https://ncert.nic.in/textbook/pdf/jehp108.pdf</t>
+        </is>
+      </c>
+      <c r="S84" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-19T01:17:12</t>
+        </is>
+      </c>
     </row>
     <row r="85">
       <c r="A85" t="inlineStr">
@@ -5272,14 +6596,32 @@
       </c>
       <c r="K85" t="inlineStr">
         <is>
-          <t>pending</t>
-        </is>
+          <t>done</t>
+        </is>
+      </c>
+      <c r="L85" t="n">
+        <v>329</v>
+      </c>
+      <c r="M85" t="n">
+        <v>16</v>
+      </c>
+      <c r="N85" t="n">
+        <v>36909</v>
+      </c>
+      <c r="O85" t="n">
+        <v>9</v>
+      </c>
+      <c r="P85" t="n">
+        <v>780.7</v>
       </c>
       <c r="Q85" t="n">
-        <v>0</v>
-      </c>
-      <c r="R85" t="inlineStr"/>
-      <c r="S85" t="inlineStr"/>
+        <v>1</v>
+      </c>
+      <c r="S85" t="inlineStr">
+        <is>
+          <t>2026-09-19T01:30:13</t>
+        </is>
+      </c>
     </row>
     <row r="86">
       <c r="A86" s="2" t="inlineStr">
@@ -5326,19 +6668,33 @@
       </c>
       <c r="K86" s="2" t="inlineStr">
         <is>
-          <t>pending</t>
-        </is>
-      </c>
-      <c r="L86" s="2" t="n"/>
-      <c r="M86" s="2" t="n"/>
-      <c r="N86" s="2" t="n"/>
-      <c r="O86" s="2" t="n"/>
-      <c r="P86" s="2" t="n"/>
+          <t>done</t>
+        </is>
+      </c>
+      <c r="L86" s="2" t="n">
+        <v>330</v>
+      </c>
+      <c r="M86" s="2" t="n">
+        <v>12</v>
+      </c>
+      <c r="N86" s="2" t="n">
+        <v>22422</v>
+      </c>
+      <c r="O86" s="2" t="n">
+        <v>4</v>
+      </c>
+      <c r="P86" s="2" t="n">
+        <v>137</v>
+      </c>
       <c r="Q86" s="2" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="R86" s="2" t="inlineStr"/>
-      <c r="S86" s="2" t="inlineStr"/>
+      <c r="S86" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-19T01:32:31</t>
+        </is>
+      </c>
     </row>
     <row r="87">
       <c r="A87" t="inlineStr">
@@ -5385,14 +6741,32 @@
       </c>
       <c r="K87" t="inlineStr">
         <is>
-          <t>pending</t>
-        </is>
+          <t>done</t>
+        </is>
+      </c>
+      <c r="L87" t="n">
+        <v>331</v>
+      </c>
+      <c r="M87" t="n">
+        <v>12</v>
+      </c>
+      <c r="N87" t="n">
+        <v>22705</v>
+      </c>
+      <c r="O87" t="n">
+        <v>17</v>
+      </c>
+      <c r="P87" t="n">
+        <v>357.2</v>
       </c>
       <c r="Q87" t="n">
-        <v>0</v>
-      </c>
-      <c r="R87" t="inlineStr"/>
-      <c r="S87" t="inlineStr"/>
+        <v>1</v>
+      </c>
+      <c r="S87" t="inlineStr">
+        <is>
+          <t>2026-09-19T01:38:29</t>
+        </is>
+      </c>
     </row>
     <row r="88">
       <c r="A88" s="2" t="inlineStr">
@@ -5439,19 +6813,33 @@
       </c>
       <c r="K88" s="2" t="inlineStr">
         <is>
-          <t>pending</t>
-        </is>
-      </c>
-      <c r="L88" s="2" t="n"/>
-      <c r="M88" s="2" t="n"/>
-      <c r="N88" s="2" t="n"/>
-      <c r="O88" s="2" t="n"/>
-      <c r="P88" s="2" t="n"/>
+          <t>done</t>
+        </is>
+      </c>
+      <c r="L88" s="2" t="n">
+        <v>332</v>
+      </c>
+      <c r="M88" s="2" t="n">
+        <v>10</v>
+      </c>
+      <c r="N88" s="2" t="n">
+        <v>18957</v>
+      </c>
+      <c r="O88" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="P88" s="2" t="n">
+        <v>133.9</v>
+      </c>
       <c r="Q88" s="2" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="R88" s="2" t="inlineStr"/>
-      <c r="S88" s="2" t="inlineStr"/>
+      <c r="S88" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-19T01:40:43</t>
+        </is>
+      </c>
     </row>
     <row r="89">
       <c r="A89" t="inlineStr">
@@ -5498,14 +6886,25 @@
       </c>
       <c r="K89" t="inlineStr">
         <is>
-          <t>pending</t>
-        </is>
+          <t>failed</t>
+        </is>
+      </c>
+      <c r="P89" t="n">
+        <v>108.9</v>
       </c>
       <c r="Q89" t="n">
-        <v>0</v>
-      </c>
-      <c r="R89" t="inlineStr"/>
-      <c r="S89" t="inlineStr"/>
+        <v>1</v>
+      </c>
+      <c r="R89" t="inlineStr">
+        <is>
+          <t>pdf fetch failed: 4 download attempts failed: HTTP 404 when fetching PDF from https://ncert.nic.in/textbook/pdf/jehp113.pdf</t>
+        </is>
+      </c>
+      <c r="S89" t="inlineStr">
+        <is>
+          <t>2026-09-19T01:42:32</t>
+        </is>
+      </c>
     </row>
   </sheetData>
   <autoFilter ref="A1:S1"/>

</xml_diff>